<commit_message>
Apply 2-day SLA completion window (created ≤ Sep 30, completed ≤ Oct 2)
Change both September reports to count tasks created through September 30 and
resolved through October 2, matching the 2-day response SLA, and set the slow
threshold to strictly > 2 days. Update the Tesorio numbers (204 completed,
1.1 d avg, 67% same-day, 38 open) and restore the deck's distribution donut and
invoices-by-portal bar charts.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nn9QKEstPX9eZ4ngSPWHBW
</commit_message>
<xml_diff>
--- a/Portal_Uploads_Report_Sep_2026.xlsx
+++ b/Portal_Uploads_Report_Sep_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Portal Uploads Report" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Data (calc)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Open &amp; In Progress" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Slow Uploads Sep - 26 (&gt;2d)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portal Uploads Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data (calc)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open &amp; In Progress" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slow Uploads Sep - 26 (&gt;2d)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -61,7 +61,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -81,6 +81,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -162,7 +167,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -245,13 +250,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -275,7 +280,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -324,7 +329,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -339,9 +344,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1344,7 +1349,7 @@
         </is>
       </c>
       <c r="K2" s="7" t="n">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="3">
@@ -5910,7 +5915,7 @@
         </is>
       </c>
       <c r="K104" s="7" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="105">
@@ -7502,7 +7507,7 @@
         </is>
       </c>
       <c r="K140" s="7" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="141">
@@ -7944,7 +7949,7 @@
         </is>
       </c>
       <c r="K150" s="7" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="151">
@@ -8300,7 +8305,7 @@
         </is>
       </c>
       <c r="K158" s="7" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="159">
@@ -9033,7 +9038,7 @@
         </is>
       </c>
       <c r="K175" s="7" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="176">
@@ -9479,7 +9484,7 @@
         </is>
       </c>
       <c r="K185" s="7" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="186">
@@ -10003,7 +10008,7 @@
         </is>
       </c>
       <c r="K197" s="7" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="198">
@@ -10040,7 +10045,7 @@
         </is>
       </c>
       <c r="K198" s="7" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="199">
@@ -10126,7 +10131,7 @@
         </is>
       </c>
       <c r="K200" s="7" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="201">
@@ -10728,7 +10733,7 @@
         </is>
       </c>
       <c r="K214" s="7" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="215">
@@ -10990,7 +10995,7 @@
         </is>
       </c>
       <c r="K220" s="7" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="221">
@@ -11387,7 +11392,7 @@
         </is>
       </c>
       <c r="K229" s="7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="230">
@@ -12140,7 +12145,7 @@
         </is>
       </c>
       <c r="K246" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="247">
@@ -12226,7 +12231,7 @@
         </is>
       </c>
       <c r="K248" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="249">
@@ -12267,7 +12272,7 @@
         </is>
       </c>
       <c r="K249" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="250">
@@ -12435,7 +12440,7 @@
         </is>
       </c>
       <c r="K253" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -12524,7 +12529,7 @@
         <v>46269.69914351852</v>
       </c>
       <c r="F4" s="18" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5">
@@ -12552,7 +12557,7 @@
         <v>46273.38089120371</v>
       </c>
       <c r="F5" s="18" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6">
@@ -12576,7 +12581,7 @@
         <v>46276.00186342592</v>
       </c>
       <c r="F6" s="18" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7">
@@ -12600,7 +12605,7 @@
         <v>46276.02268518518</v>
       </c>
       <c r="F7" s="18" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8">
@@ -12628,7 +12633,7 @@
         <v>46276.64129629629</v>
       </c>
       <c r="F8" s="18" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
@@ -12656,7 +12661,7 @@
         <v>46282.87568287037</v>
       </c>
       <c r="F9" s="18" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
@@ -12684,7 +12689,7 @@
         <v>46286.39118055555</v>
       </c>
       <c r="F10" s="18" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11">
@@ -12712,7 +12717,7 @@
         <v>46288.36726851852</v>
       </c>
       <c r="F11" s="18" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
@@ -12740,7 +12745,7 @@
         <v>46294.65384259259</v>
       </c>
       <c r="F12" s="19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -12768,7 +12773,7 @@
         <v>46294.6583912037</v>
       </c>
       <c r="F13" s="19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -12796,7 +12801,7 @@
         <v>46294.66214120371</v>
       </c>
       <c r="F14" s="19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -12824,7 +12829,7 @@
         <v>46295.48530092592</v>
       </c>
       <c r="F15" s="19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>